<commit_message>
Update course games and media handling
Integrate workbook-backed vocabulary and quiz games, improve game flows, and update asset delivery and deployment support.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/static/data/tests.xlsx
+++ b/static/data/tests.xlsx
@@ -5,23 +5,24 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aca0a008a5ddf25f/course_app/static/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ACA0A008A5DDF25F/course_app/static/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="11_423C6FE1565BEAFEE87DD0355E5DCE3AA7C98B74" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{293A9247-CF8C-41DE-9053-9BD14D633900}"/>
+  <xr:revisionPtr revIDLastSave="198" documentId="11_423C6FE1565BEAFEE87DD0355E5DCE3AA7C98B74" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A167B41-D4D5-4042-BDDB-43B0B8D0061D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="English Test" sheetId="1" r:id="rId1"/>
-    <sheet name="test_each_every" sheetId="2" r:id="rId2"/>
+    <sheet name="Each vs Every" sheetId="2" r:id="rId2"/>
+    <sheet name="Directions" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1201" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="430">
   <si>
     <t>Question #</t>
   </si>
@@ -1257,13 +1258,67 @@
   </si>
   <si>
     <t>b</t>
+  </si>
+  <si>
+    <t>multiple choice</t>
+  </si>
+  <si>
+    <t>gammar</t>
+  </si>
+  <si>
+    <t>north</t>
+  </si>
+  <si>
+    <t>south</t>
+  </si>
+  <si>
+    <t>east</t>
+  </si>
+  <si>
+    <t>west</t>
+  </si>
+  <si>
+    <t>The sun rises in the __________</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The sun sets in the __________</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> If you travel from Mexico to Canada, you go __________</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> If you travel from Canada to Mexico, you go __________</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Florida is east of California, so California is __________ of Florida</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> New York is on the __________ coast of the United States</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> California is on the __________ coast of the United States</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> A compass needle usually points __________</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> If you go south and then turn around, you are going __________</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Japan is __________ of China</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>compass points</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1276,6 +1331,25 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1292,7 +1366,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1300,11 +1374,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1318,11 +1401,1338 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="94">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F4E78"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F4E78"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F4E78"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F4E78"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F4E78"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F4E78"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1377,53 +2787,10 @@
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Calibri"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF1F4E78"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Table Style 1" pivot="0" count="0" xr9:uid="{E1D4C594-9A57-434F-A331-6E1590A588C7}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1435,41 +2802,137 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6309D6D7-6C25-4AAD-A555-A6D2DEF6ED12}" name="test_final" displayName="test_final" ref="F1:K101" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6309D6D7-6C25-4AAD-A555-A6D2DEF6ED12}" name="test_final" displayName="test_final" ref="F1:K101" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
   <autoFilter ref="F1:K101" xr:uid="{6309D6D7-6C25-4AAD-A555-A6D2DEF6ED12}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{96F3B88C-0411-440D-AF54-574779021F94}" name="Question" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{EBBAA3D2-1BFC-4700-8AE9-A392532D2E00}" name="Answer A" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{3ED6B182-8051-4120-ABA6-927612AF6D5D}" name="Answer B" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{802D0621-8FC6-4679-BFE1-CE8460F49AE7}" name="Answer C" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{EE87AA6D-D5DA-4245-9C89-E8CA48053929}" name="Answer D" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{E6B8761B-94ED-45DF-AE39-A1D83B30B846}" name="Correct Answer" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{96F3B88C-0411-440D-AF54-574779021F94}" name="Question" dataDxfId="80"/>
+    <tableColumn id="2" xr3:uid="{EBBAA3D2-1BFC-4700-8AE9-A392532D2E00}" name="Answer A" dataDxfId="79"/>
+    <tableColumn id="3" xr3:uid="{3ED6B182-8051-4120-ABA6-927612AF6D5D}" name="Answer B" dataDxfId="78"/>
+    <tableColumn id="4" xr3:uid="{802D0621-8FC6-4679-BFE1-CE8460F49AE7}" name="Answer C" dataDxfId="77"/>
+    <tableColumn id="5" xr3:uid="{EE87AA6D-D5DA-4245-9C89-E8CA48053929}" name="Answer D" dataDxfId="76"/>
+    <tableColumn id="6" xr3:uid="{E6B8761B-94ED-45DF-AE39-A1D83B30B846}" name="Correct Answer" dataDxfId="75"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D9E92822-8E44-4295-A523-2912204D62A5}" name="test_each_every" displayName="test_each_every" ref="A1:J21" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D9E92822-8E44-4295-A523-2912204D62A5}" name="test_each_every" displayName="test_each_every" ref="A1:J21" totalsRowShown="0" headerRowDxfId="93" dataDxfId="92">
   <autoFilter ref="A1:J21" xr:uid="{D9E92822-8E44-4295-A523-2912204D62A5}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{3D83272E-A050-4FDE-BEBC-D8087B7E8E45}" name="Question #" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{9B00EA2B-4C93-4758-8F20-02E51FEA14C6}" name="Question Type" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{AA1900C6-C3C4-4027-87CA-684D62ACF597}" name="Difficulty Level" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{11623D33-1546-4E2C-8F29-F4665AF2A0CB}" name="Category" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{FF0C83A8-EC90-4D3F-B587-88BCB04F714E}" name="Part of Speech Being Tested" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{3D83272E-A050-4FDE-BEBC-D8087B7E8E45}" name="Question #" dataDxfId="91"/>
+    <tableColumn id="2" xr3:uid="{9B00EA2B-4C93-4758-8F20-02E51FEA14C6}" name="Question Type" dataDxfId="90"/>
+    <tableColumn id="3" xr3:uid="{AA1900C6-C3C4-4027-87CA-684D62ACF597}" name="Difficulty Level" dataDxfId="89"/>
+    <tableColumn id="4" xr3:uid="{11623D33-1546-4E2C-8F29-F4665AF2A0CB}" name="Category" dataDxfId="88"/>
+    <tableColumn id="5" xr3:uid="{FF0C83A8-EC90-4D3F-B587-88BCB04F714E}" name="Part of Speech Being Tested" dataDxfId="87"/>
     <tableColumn id="6" xr3:uid="{CBE3F450-4650-4208-9C2E-4FB33B20B8F3}" name="Question"/>
-    <tableColumn id="7" xr3:uid="{65C3CC17-F974-433D-B91A-C02EEF5BC72D}" name="Answer A" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{8E79768C-6CE4-49DF-BF5B-A0181F789000}" name="Answer B" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{AA1603D8-C236-491D-B67E-2CE3C78CFB12}" name="Answer C" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{9F898204-48F2-44FC-863C-9A53A353B888}" name="Correct Answer" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{65C3CC17-F974-433D-B91A-C02EEF5BC72D}" name="Answer A" dataDxfId="86"/>
+    <tableColumn id="8" xr3:uid="{8E79768C-6CE4-49DF-BF5B-A0181F789000}" name="Answer B" dataDxfId="85"/>
+    <tableColumn id="9" xr3:uid="{AA1603D8-C236-491D-B67E-2CE3C78CFB12}" name="Answer C" dataDxfId="84"/>
+    <tableColumn id="11" xr3:uid="{9F898204-48F2-44FC-863C-9A53A353B888}" name="Correct Answer" dataDxfId="83"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6ADE9DE9-EB19-4334-AD50-60179D57A717}" name="Table1" displayName="Table1" ref="A1:K11" totalsRowShown="0" headerRowDxfId="60" dataDxfId="61" headerRowBorderDxfId="73" tableBorderDxfId="74">
+  <autoFilter ref="A1:K11" xr:uid="{6ADE9DE9-EB19-4334-AD50-60179D57A717}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{5E649DB3-771A-4365-9412-B78AC68B96D8}" name="Question #" dataDxfId="72"/>
+    <tableColumn id="2" xr3:uid="{63D65448-BD5B-477A-924D-0DC965964A36}" name="Question Type" dataDxfId="71"/>
+    <tableColumn id="3" xr3:uid="{99B1B685-4D47-4FDC-B648-7C94FC5835B8}" name="Difficulty Level" dataDxfId="70"/>
+    <tableColumn id="4" xr3:uid="{83C7BCA2-9428-4EEF-80D6-E6FC17DF3E0A}" name="Category" dataDxfId="69"/>
+    <tableColumn id="5" xr3:uid="{72E939C9-7E4E-4F01-B3D9-FE903C0C4555}" name="Part of Speech Being Tested" dataDxfId="68"/>
+    <tableColumn id="6" xr3:uid="{123F0C65-A39C-4FCC-88BA-4EA706819B03}" name="Question" dataDxfId="67"/>
+    <tableColumn id="7" xr3:uid="{D65BD10D-542E-4FB5-8942-88BC30A6CAEE}" name="Answer A" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{63527AC9-CB42-492B-9862-7DC562A6CE33}" name="Answer B" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{4E9D1A44-927A-4F80-A109-F6A27148BAC2}" name="Answer C" dataDxfId="64"/>
+    <tableColumn id="10" xr3:uid="{A7F19DFB-D6FB-437C-9EDA-F5D05A167E4D}" name="Answer D" dataDxfId="63"/>
+    <tableColumn id="11" xr3:uid="{B21EFB41-6350-4299-B602-68B8825B6791}" name="Correct Answer" dataDxfId="62"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4291E79C-4F34-4FC5-8649-4B62121E46E1}" name="Table15" displayName="Table15" ref="A13:K23" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58" headerRowBorderDxfId="56" tableBorderDxfId="57">
+  <autoFilter ref="A13:K23" xr:uid="{4291E79C-4F34-4FC5-8649-4B62121E46E1}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{D3406167-53ED-4CAF-B949-26F46D5BB710}" name="Question #" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{D371F9DE-7151-468A-96B9-E7E4C6B650B9}" name="Question Type" dataDxfId="54"/>
+    <tableColumn id="3" xr3:uid="{6E4792AD-B33B-44D6-A7A6-EA28B91DE2A1}" name="Difficulty Level" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{9C389DF7-A309-43B7-AD6D-1EBB2D151C8C}" name="Category" dataDxfId="52"/>
+    <tableColumn id="5" xr3:uid="{4D745F0A-F7D4-4A71-B8B5-A647B695D4D1}" name="Part of Speech Being Tested" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{7CD3E898-DC19-4665-9FB9-57DD566F80D9}" name="Question" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{3FC6CA46-2AFC-4AF2-BE10-719D627E72D0}" name="Answer A" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{71FF56DD-1017-48FE-8E3A-6B1BBD25D4B8}" name="Answer B" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{14AE869D-E3D5-4BFC-8326-6C555FF642E6}" name="Answer C" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{DCFFF722-14C9-40A9-B103-B1CC6E55154E}" name="Answer D" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{7DD65614-F877-44D0-B4EC-FAF28608F495}" name="Correct Answer" dataDxfId="49"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{345BC960-40E4-41EA-A74F-20EB5CD35603}" name="Table16" displayName="Table16" ref="A25:K35" totalsRowShown="0" headerRowDxfId="48" dataDxfId="47" headerRowBorderDxfId="45" tableBorderDxfId="46">
+  <autoFilter ref="A25:K35" xr:uid="{345BC960-40E4-41EA-A74F-20EB5CD35603}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{3D228515-3382-4730-9BE6-137DBB27B08A}" name="Question #" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{00F117CF-458E-4A12-92D3-574FA5D67B3A}" name="Question Type" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{2D4CAC6C-7B35-4DFB-A062-5C7750F16C62}" name="Difficulty Level" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{3E929698-2ACA-41E1-8A35-70D90032E273}" name="Category" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{AC93A8D1-39A7-4F43-8F18-0B67AB2D3F2D}" name="Part of Speech Being Tested" dataDxfId="40"/>
+    <tableColumn id="6" xr3:uid="{3DC2A1A4-E507-4614-BAB2-5EBBF6B3A37F}" name="Question" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{5458B80C-1532-4FA3-8172-580CC148011A}" name="Answer A" dataDxfId="38"/>
+    <tableColumn id="8" xr3:uid="{1C107A13-320C-4CC3-9D13-AAABC06B12D1}" name="Answer B" dataDxfId="37"/>
+    <tableColumn id="9" xr3:uid="{A423EF32-42AB-48CA-816D-D6FC0330BBCD}" name="Answer C" dataDxfId="36"/>
+    <tableColumn id="10" xr3:uid="{4CD6F68A-85C8-4BCD-9004-18FC2C879334}" name="Answer D" dataDxfId="35"/>
+    <tableColumn id="11" xr3:uid="{01E83D48-5ED1-4BD5-8CE1-1F8C69CFB3B8}" name="Correct Answer" dataDxfId="34"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{65B034F6-B042-421B-BDA7-3FAC3ED8B9FF}" name="Table17" displayName="Table17" ref="A37:K47" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32" headerRowBorderDxfId="30" tableBorderDxfId="31">
+  <autoFilter ref="A37:K47" xr:uid="{65B034F6-B042-421B-BDA7-3FAC3ED8B9FF}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{8223C20B-51AA-4496-B0BA-47D975D0C607}" name="Question #" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{3634F27B-12ED-410A-86E3-E970704E2F5F}" name="Question Type" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{761884F9-7D1B-44FB-A609-674FD4A2A11C}" name="Difficulty Level" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{6D49156E-0908-44C9-9B6B-E3723E1C24C6}" name="Category" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{E85ED647-287D-4682-A215-D039EEAC94DD}" name="Part of Speech Being Tested" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{2EBDCFFE-D7E2-4497-B9B1-F91139F045AA}" name="Question" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{DA6C2F7A-E785-4262-B3E9-21BE049F09DD}" name="Answer A" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{97747325-DBA5-4615-9E6E-656E1C7224D7}" name="Answer B" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{A339B994-55BD-460C-8406-16AA04AE9A37}" name="Answer C" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{F4D85831-33B0-4952-B53A-B5F8F2422695}" name="Answer D" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{14AEBA91-6CB5-45A9-BAEB-F3B384BBC0B3}" name="Correct Answer" dataDxfId="19"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{4E8C8CE0-E970-4413-AA8C-3FD39027A767}" name="Table18" displayName="Table18" ref="A49:K59" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17" headerRowBorderDxfId="15" tableBorderDxfId="16">
+  <autoFilter ref="A49:K59" xr:uid="{4E8C8CE0-E970-4413-AA8C-3FD39027A767}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{80BED708-8617-46E5-9D84-23F771D0D154}" name="Question #" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{399B23E0-8920-4499-B9D1-8279EF3D8BFC}" name="Question Type" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{CA26D08C-E153-45CB-AB34-1D30D0988B55}" name="Difficulty Level" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{FCA29918-5BF0-4AB0-A8EC-F249BCE0CD19}" name="Category" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{98569F19-0FDC-4C12-99B0-50433AEC7013}" name="Part of Speech Being Tested" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{95C6C488-7A6D-4733-A991-E084D57E345E}" name="Question" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{DF8CAFB0-3A72-4716-A4B7-34CBA7F292B3}" name="Answer A" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{2D2F41C0-ABB0-4993-B161-3784E4722126}" name="Answer B" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{127E11C4-5E9B-4AFA-A31E-6152B597925F}" name="Answer C" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{CFA4B1C1-04CD-44C0-B536-CA0BC1A4F5D2}" name="Answer D" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{C6FD9A5C-9186-427C-9923-D27A249F9B9D}" name="Correct Answer" dataDxfId="4"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -5517,7 +6980,7 @@
         <v>408</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -5549,7 +7012,7 @@
         <v>408</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -5581,7 +7044,7 @@
         <v>408</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -6006,4 +7469,1941 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8242DB64-573F-4995-86F6-9CA33553B29D}">
+  <dimension ref="A1:O59"/>
+  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.44140625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.88671875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="11" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.109375" style="6" customWidth="1"/>
+    <col min="6" max="6" width="42.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" style="6" customWidth="1"/>
+    <col min="8" max="9" width="9.21875" style="6" customWidth="1"/>
+    <col min="10" max="10" width="9.44140625" style="6" customWidth="1"/>
+    <col min="11" max="11" width="13.21875" style="6" customWidth="1"/>
+    <col min="12" max="14" width="8.88671875" style="6"/>
+    <col min="15" max="16" width="19.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="36.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="42.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="37.21875" style="6" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="37.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="28.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="42" style="6" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="25" max="16384" width="8.88671875" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="12" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>424</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="6">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="O10" s="5"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="6">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="12" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="6">
+        <v>1</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="6">
+        <v>2</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="6">
+        <v>3</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="6">
+        <v>4</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="6">
+        <v>5</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="6">
+        <v>6</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="6">
+        <v>7</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="6">
+        <v>8</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="6">
+        <v>9</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="6">
+        <v>10</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="12" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="6">
+        <v>1</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="6">
+        <v>2</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="6">
+        <v>3</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="6">
+        <v>4</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="6">
+        <v>5</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="6">
+        <v>6</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="6">
+        <v>7</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>424</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="6">
+        <v>8</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="6">
+        <v>9</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="6">
+        <v>10</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="12" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I37" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J37" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="K37" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="6">
+        <v>1</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" s="6">
+        <v>2</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="6">
+        <v>3</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J40" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="6">
+        <v>4</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="6">
+        <v>5</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I42" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J42" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K42" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="6">
+        <v>6</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I43" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="6">
+        <v>7</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>424</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J44" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" s="6">
+        <v>8</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K45" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="6">
+        <v>9</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I46" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J46" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K46" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" s="6">
+        <v>10</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="12" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G49" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H49" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I49" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J49" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="K49" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" s="6">
+        <v>1</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="G50" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I50" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J50" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K50" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" s="6">
+        <v>2</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I51" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J51" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K51" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" s="6">
+        <v>3</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J52" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K52" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="6">
+        <v>4</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F53" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="G53" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H53" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I53" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J53" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K53" s="6" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" s="6">
+        <v>5</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I54" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J54" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K54" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="6">
+        <v>6</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I55" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J55" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K55" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" s="6">
+        <v>7</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>424</v>
+      </c>
+      <c r="G56" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I56" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J56" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K56" s="6" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" s="6">
+        <v>8</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="G57" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H57" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I57" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J57" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K57" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" s="6">
+        <v>9</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H58" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I58" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J58" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K58" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" s="6">
+        <v>10</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="I59" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="J59" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K59" s="6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="5">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>